<commit_message>
docs: cover Developer support lifecycle and guarded Undo in acceptance
</commit_message>
<xml_diff>
--- a/docs/acceptance/PAWS_TESTING_MANUAL_ACCEPTANCE.xlsx
+++ b/docs/acceptance/PAWS_TESTING_MANUAL_ACCEPTANCE.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Acceptance" sheetId="1" r:id="R79ce90a018864268"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Acceptance" sheetId="1" r:id="Rf2717e40b7ac499f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -152,8 +152,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PawsManualAcceptance" displayName="PawsManualAcceptance" ref="A8:M143" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A8:M143"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PawsManualAcceptance" displayName="PawsManualAcceptance" ref="A8:M149" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A8:M149"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Feature"/>
@@ -483,41 +483,41 @@
         <x:v>Cases</x:v>
       </x:c>
       <x:c r="B6" s="1" t="n">
-        <x:v>135</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C6" s="1" t="str">
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D6" s="1" t="n">
-        <x:f>COUNTIFS(H9:H143,"Pass")</x:f>
+        <x:f>COUNTIFS(H9:H149,"Pass")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="1" t="str">
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="F6" s="1" t="n">
-        <x:f>COUNTIFS(H9:H143,"Fail")</x:f>
+        <x:f>COUNTIFS(H9:H149,"Fail")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G6" s="1" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H6" s="1" t="n">
-        <x:f>COUNTIFS(H9:H143,"Blocked")</x:f>
+        <x:f>COUNTIFS(H9:H149,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="1" t="str">
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="J6" s="1" t="n">
-        <x:f>COUNTIFS(H9:H143,"Not run")</x:f>
-        <x:v>135</x:v>
+        <x:f>COUNTIFS(H9:H149,"Not run")</x:f>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="K6" s="1" t="str">
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="L6" s="1" t="n">
-        <x:f>COUNTIFS(H9:H143,"N/A")</x:f>
+        <x:f>COUNTIFS(H9:H149,"N/A")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="1"/>
@@ -5033,6 +5033,204 @@
         <x:v>Not executable on the cloud-free Pages frontend.</x:v>
       </x:c>
     </x:row>
+    <x:row r="144" ht="60" customHeight="1">
+      <x:c r="A144" s="9" t="str">
+        <x:v>SUP-01</x:v>
+      </x:c>
+      <x:c r="B144" s="9" t="str">
+        <x:v>Developer support sessions</x:v>
+      </x:c>
+      <x:c r="C144" s="9" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="D144" s="9" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E144" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F144" s="9" t="str">
+        <x:v>Choose an active synthetic target account, submit a blank/oversized reason, then start with a valid reason.</x:v>
+      </x:c>
+      <x:c r="G144" s="9" t="str">
+        <x:v>Reason is required and bounded; only an active supported target starts a30-minute context with the real Developer actor retained.</x:v>
+      </x:c>
+      <x:c r="H144" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I144" s="12" t="str"/>
+      <x:c r="J144" s="12" t="str"/>
+      <x:c r="K144" s="12" t="str"/>
+      <x:c r="L144" s="13"/>
+      <x:c r="M144" s="9" t="str">
+        <x:v>Developer support adapter/backend required; Demo role switching is not equivalent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="60" customHeight="1">
+      <x:c r="A145" s="9" t="str">
+        <x:v>SUP-02</x:v>
+      </x:c>
+      <x:c r="B145" s="9" t="str">
+        <x:v>Developer support sessions</x:v>
+      </x:c>
+      <x:c r="C145" s="9" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="D145" s="9" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E145" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F145" s="9" t="str">
+        <x:v>Inspect the support banner and perform an allowed synthetic edit, then inspect recent operations and audit.</x:v>
+      </x:c>
+      <x:c r="G145" s="9" t="str">
+        <x:v>Target context is clear, actions are real in that environment, and actor/target/reason/change capture are attributable without identity transfer.</x:v>
+      </x:c>
+      <x:c r="H145" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I145" s="12" t="str"/>
+      <x:c r="J145" s="12" t="str"/>
+      <x:c r="K145" s="12" t="str"/>
+      <x:c r="L145" s="13"/>
+      <x:c r="M145" s="9" t="str">
+        <x:v>Use disposable backend records only; never real staff data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="60" customHeight="1">
+      <x:c r="A146" s="9" t="str">
+        <x:v>SUP-03</x:v>
+      </x:c>
+      <x:c r="B146" s="9" t="str">
+        <x:v>Developer support sessions</x:v>
+      </x:c>
+      <x:c r="C146" s="9" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="D146" s="9" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E146" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F146" s="9" t="str">
+        <x:v>Select Return to myself, reload and inspect subsequent requests and private views.</x:v>
+      </x:c>
+      <x:c r="G146" s="9" t="str">
+        <x:v>Context ends and support headers/cached target data clear; subsequent actions use the Developer's own identity.</x:v>
+      </x:c>
+      <x:c r="H146" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I146" s="12" t="str"/>
+      <x:c r="J146" s="12" t="str"/>
+      <x:c r="K146" s="12" t="str"/>
+      <x:c r="L146" s="13"/>
+      <x:c r="M146" s="9" t="str">
+        <x:v>Ending an already ended context must not reopen it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147" ht="60" customHeight="1">
+      <x:c r="A147" s="9" t="str">
+        <x:v>SUP-04</x:v>
+      </x:c>
+      <x:c r="B147" s="9" t="str">
+        <x:v>Developer support sessions</x:v>
+      </x:c>
+      <x:c r="C147" s="9" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="D147" s="9" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E147" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F147" s="9" t="str">
+        <x:v>Expire the context at30minutes, disable the target or require its password change, then retry a supported action.</x:v>
+      </x:c>
+      <x:c r="G147" s="9" t="str">
+        <x:v>Expired/ended/unavailable targets fail closed; stale tabs cannot keep acting as the target.</x:v>
+      </x:c>
+      <x:c r="H147" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I147" s="12" t="str"/>
+      <x:c r="J147" s="12" t="str"/>
+      <x:c r="K147" s="12" t="str"/>
+      <x:c r="L147" s="13"/>
+      <x:c r="M147" s="9" t="str">
+        <x:v>Use controlled expiry and target fixtures, not production account edits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148" ht="60" customHeight="1">
+      <x:c r="A148" s="9" t="str">
+        <x:v>SUP-05</x:v>
+      </x:c>
+      <x:c r="B148" s="9" t="str">
+        <x:v>Developer support sessions</x:v>
+      </x:c>
+      <x:c r="C148" s="9" t="str">
+        <x:v>Developer</x:v>
+      </x:c>
+      <x:c r="D148" s="9" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E148" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F148" s="9" t="str">
+        <x:v>Undo a captured own operation without a later change; repeat Undo and try another with a conflicting later edit.</x:v>
+      </x:c>
+      <x:c r="G148" s="9" t="str">
+        <x:v>Valid Undo restores only captured data once; conflict/foreign operation is refused and later edits/audit history remain.</x:v>
+      </x:c>
+      <x:c r="H148" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I148" s="12" t="str"/>
+      <x:c r="J148" s="12" t="str"/>
+      <x:c r="K148" s="12" t="str"/>
+      <x:c r="L148" s="13"/>
+      <x:c r="M148" s="9" t="str">
+        <x:v>Actual version/transaction/recovery evidence required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="60" customHeight="1">
+      <x:c r="A149" s="9" t="str">
+        <x:v>SUP-06</x:v>
+      </x:c>
+      <x:c r="B149" s="9" t="str">
+        <x:v>Developer support sessions</x:v>
+      </x:c>
+      <x:c r="C149" s="9" t="str">
+        <x:v>Faculty / Administrator / Developer</x:v>
+      </x:c>
+      <x:c r="D149" s="9" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E149" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F149" s="9" t="str">
+        <x:v>Try non-Developer start/list/end/Undo, a foreign context ID and unsupported support routes such as protected artifacts.</x:v>
+      </x:c>
+      <x:c r="G149" s="9" t="str">
+        <x:v>Authority denies non-Developer/foreign-context or restricted-route access; support is not a blanket data/download bypass.</x:v>
+      </x:c>
+      <x:c r="H149" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I149" s="12" t="str"/>
+      <x:c r="J149" s="12" t="str"/>
+      <x:c r="K149" s="12" t="str"/>
+      <x:c r="L149" s="13"/>
+      <x:c r="M149" s="9" t="str">
+        <x:v>server/src/support/support-service.js is the ported contract.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:M2"/>
@@ -5044,7 +5242,7 @@
     <x:mergeCell ref="K4:M4"/>
     <x:mergeCell ref="A5:M5"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="H9:H143">
+  <x:conditionalFormatting sqref="H9:H149">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <x:formula>"Fail"</x:formula>
     </x:cfRule>
@@ -5059,13 +5257,13 @@
     <x:dataValidation type="list" sqref="H3">
       <x:formula1>"Frontend Demo,Firebase Lab,Isolated backend"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="H9:H143">
+    <x:dataValidation type="list" sqref="H9:H149">
       <x:formula1>"Not run,Pass,Fail,Blocked,N/A"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7dbd17e669b42b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6d461a73621460b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: complete Scheduling Tasks and Testing identity acceptance coverage
</commit_message>
<xml_diff>
--- a/docs/acceptance/PAWS_TESTING_MANUAL_ACCEPTANCE.xlsx
+++ b/docs/acceptance/PAWS_TESTING_MANUAL_ACCEPTANCE.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Acceptance" sheetId="1" r:id="Rf2717e40b7ac499f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Acceptance" sheetId="1" r:id="R4efff5ecc2b2469c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5263,7 +5263,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6d461a73621460b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe571fc527ac415f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: synchronize complete148-case manual acceptance catalog
</commit_message>
<xml_diff>
--- a/docs/acceptance/PAWS_TESTING_MANUAL_ACCEPTANCE.xlsx
+++ b/docs/acceptance/PAWS_TESTING_MANUAL_ACCEPTANCE.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Acceptance" sheetId="1" r:id="R4efff5ecc2b2469c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Acceptance" sheetId="1" r:id="R4240cc01516d4050"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -152,8 +152,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PawsManualAcceptance" displayName="PawsManualAcceptance" ref="A8:M149" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A8:M149"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PawsManualAcceptance" displayName="PawsManualAcceptance" ref="A8:M156" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A8:M156"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Feature"/>
@@ -483,41 +483,41 @@
         <x:v>Cases</x:v>
       </x:c>
       <x:c r="B6" s="1" t="n">
-        <x:v>141</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="C6" s="1" t="str">
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="D6" s="1" t="n">
-        <x:f>COUNTIFS(H9:H149,"Pass")</x:f>
+        <x:f>COUNTIFS(H9:H156,"Pass")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="1" t="str">
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="F6" s="1" t="n">
-        <x:f>COUNTIFS(H9:H149,"Fail")</x:f>
+        <x:f>COUNTIFS(H9:H156,"Fail")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G6" s="1" t="str">
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="H6" s="1" t="n">
-        <x:f>COUNTIFS(H9:H149,"Blocked")</x:f>
+        <x:f>COUNTIFS(H9:H156,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="1" t="str">
         <x:v>Not run</x:v>
       </x:c>
       <x:c r="J6" s="1" t="n">
-        <x:f>COUNTIFS(H9:H149,"Not run")</x:f>
-        <x:v>141</x:v>
+        <x:f>COUNTIFS(H9:H156,"Not run")</x:f>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="K6" s="1" t="str">
         <x:v>N/A</x:v>
       </x:c>
       <x:c r="L6" s="1" t="n">
-        <x:f>COUNTIFS(H9:H149,"N/A")</x:f>
+        <x:f>COUNTIFS(H9:H156,"N/A")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="1"/>
@@ -5231,6 +5231,237 @@
         <x:v>server/src/support/support-service.js is the ported contract.</x:v>
       </x:c>
     </x:row>
+    <x:row r="150" ht="60" customHeight="1">
+      <x:c r="A150" s="9" t="str">
+        <x:v>TSK-01</x:v>
+      </x:c>
+      <x:c r="B150" s="9" t="str">
+        <x:v>Scheduling Tasks queue</x:v>
+      </x:c>
+      <x:c r="C150" s="9" t="str">
+        <x:v>Administrator / Faculty</x:v>
+      </x:c>
+      <x:c r="D150" s="9" t="str">
+        <x:v>D/B</x:v>
+      </x:c>
+      <x:c r="E150" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F150" s="9" t="str">
+        <x:v>Open Calendar Tasks, inspect every available task category and combine year, course, faculty, date, undated and review-status filters.</x:v>
+      </x:c>
+      <x:c r="G150" s="9" t="str">
+        <x:v>Only authorized tasks and counts appear; missing assignments and undated issues remain explicit; pagination does not duplicate or omit records.</x:v>
+      </x:c>
+      <x:c r="H150" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I150" s="12" t="str"/>
+      <x:c r="J150" s="12" t="str"/>
+      <x:c r="K150" s="12" t="str"/>
+      <x:c r="L150" s="13"/>
+      <x:c r="M150" s="9" t="str">
+        <x:v>server/src/scheduling/scheduling-task-api.js and repository are the contract.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="60" customHeight="1">
+      <x:c r="A151" s="9" t="str">
+        <x:v>TSK-02</x:v>
+      </x:c>
+      <x:c r="B151" s="9" t="str">
+        <x:v>Scheduling Tasks queue</x:v>
+      </x:c>
+      <x:c r="C151" s="9" t="str">
+        <x:v>Administrator</x:v>
+      </x:c>
+      <x:c r="D151" s="9" t="str">
+        <x:v>D/B</x:v>
+      </x:c>
+      <x:c r="E151" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F151" s="9" t="str">
+        <x:v>Mark an eligible current task reviewed, reopen it if supported, and repeat with the review-write gate off.</x:v>
+      </x:c>
+      <x:c r="G151" s="9" t="str">
+        <x:v>Only the supported current-version review transition saves; disabled writes remain disabled; reviewing does not silently alter the timetable.</x:v>
+      </x:c>
+      <x:c r="H151" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I151" s="12" t="str"/>
+      <x:c r="J151" s="12" t="str"/>
+      <x:c r="K151" s="12" t="str"/>
+      <x:c r="L151" s="13"/>
+      <x:c r="M151" s="9" t="str">
+        <x:v>Demo ALL_WRITES cannot certify actual backend gate state.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="60" customHeight="1">
+      <x:c r="A152" s="9" t="str">
+        <x:v>TSK-03</x:v>
+      </x:c>
+      <x:c r="B152" s="9" t="str">
+        <x:v>Scheduling Tasks queue</x:v>
+      </x:c>
+      <x:c r="C152" s="9" t="str">
+        <x:v>Faculty / Administrator</x:v>
+      </x:c>
+      <x:c r="D152" s="9" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E152" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F152" s="9" t="str">
+        <x:v>Attempt an unauthorized review and a review using a stale task/source version after another edit.</x:v>
+      </x:c>
+      <x:c r="G152" s="9" t="str">
+        <x:v>Authority rejects unauthorized or stale actions and asks for refresh rather than falsely reporting completion.</x:v>
+      </x:c>
+      <x:c r="H152" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I152" s="12" t="str"/>
+      <x:c r="J152" s="12" t="str"/>
+      <x:c r="K152" s="12" t="str"/>
+      <x:c r="L152" s="13"/>
+      <x:c r="M152" s="9" t="str">
+        <x:v>Requires trusted identity and source-version recheck.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="60" customHeight="1">
+      <x:c r="A153" s="9" t="str">
+        <x:v>TSK-04</x:v>
+      </x:c>
+      <x:c r="B153" s="9" t="str">
+        <x:v>Scheduling Tasks queue</x:v>
+      </x:c>
+      <x:c r="C153" s="9" t="str">
+        <x:v>Reviewer</x:v>
+      </x:c>
+      <x:c r="D153" s="9" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E153" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F153" s="9" t="str">
+        <x:v>Use the empty-to-assigned-to-empty fixture from TA-04, including an Undo, then reload reviewed tasks.</x:v>
+      </x:c>
+      <x:c r="G153" s="9" t="str">
+        <x:v>Assignment version changes invalidate the prior review even if values return to empty; task state matches the current source.</x:v>
+      </x:c>
+      <x:c r="H153" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I153" s="12" t="str"/>
+      <x:c r="J153" s="12" t="str"/>
+      <x:c r="K153" s="12" t="str"/>
+      <x:c r="L153" s="13"/>
+      <x:c r="M153" s="9" t="str">
+        <x:v>Verify the actual version-trigger/ABA behavior, not just a browser badge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="60" customHeight="1">
+      <x:c r="A154" s="9" t="str">
+        <x:v>ACC-07</x:v>
+      </x:c>
+      <x:c r="B154" s="9" t="str">
+        <x:v>Accounts and effective access</x:v>
+      </x:c>
+      <x:c r="C154" s="9" t="str">
+        <x:v>Owner</x:v>
+      </x:c>
+      <x:c r="D154" s="9" t="str">
+        <x:v>D/L</x:v>
+      </x:c>
+      <x:c r="E154" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F154" s="9" t="str">
+        <x:v>In the older Testing account form, preview bulk provisioning with missing/duplicate email and orphaned-auth fixtures, then change source data before apply.</x:v>
+      </x:c>
+      <x:c r="G154" s="9" t="str">
+        <x:v>Invalid/ambiguous identities are excluded for review; stale preview refuses apply; unsupported SQL role cleanup is explicitly refused.</x:v>
+      </x:c>
+      <x:c r="H154" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I154" s="12" t="str"/>
+      <x:c r="J154" s="12" t="str"/>
+      <x:c r="K154" s="12" t="str"/>
+      <x:c r="L154" s="13"/>
+      <x:c r="M154" s="9" t="str">
+        <x:v>Legacy Testing form; not the PR148 SQL-authoritative account contract.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="60" customHeight="1">
+      <x:c r="A155" s="9" t="str">
+        <x:v>ACC-08</x:v>
+      </x:c>
+      <x:c r="B155" s="9" t="str">
+        <x:v>Accounts and effective access</x:v>
+      </x:c>
+      <x:c r="C155" s="9" t="str">
+        <x:v>Owner / new Faculty</x:v>
+      </x:c>
+      <x:c r="D155" s="9" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="E155" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F155" s="9" t="str">
+        <x:v>Provision only approved synthetic Lab accounts from a current preview and inspect partial failures, required password change and cleared temporary-password fields.</x:v>
+      </x:c>
+      <x:c r="G155" s="9" t="str">
+        <x:v>Counts and linked profiles agree with real Auth; initial password-change policy holds; failures are recoverable and no credential enters logs/history/exports.</x:v>
+      </x:c>
+      <x:c r="H155" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I155" s="12" t="str"/>
+      <x:c r="J155" s="12" t="str"/>
+      <x:c r="K155" s="12" t="str"/>
+      <x:c r="L155" s="13"/>
+      <x:c r="M155" s="9" t="str">
+        <x:v>Real Lab provisioning only when explicitly authorized; Demo accounts are simulated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="60" customHeight="1">
+      <x:c r="A156" s="9" t="str">
+        <x:v>AUTH-09</x:v>
+      </x:c>
+      <x:c r="B156" s="9" t="str">
+        <x:v>Authentication and session</x:v>
+      </x:c>
+      <x:c r="C156" s="9" t="str">
+        <x:v>Synthetic phone user</x:v>
+      </x:c>
+      <x:c r="D156" s="9" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="E156" s="9" t="str">
+        <x:v>Synthetic fixtures; selected mode and SHA recorded; required role available.</x:v>
+      </x:c>
+      <x:c r="F156" s="9" t="str">
+        <x:v>Where enabled, exercise phone/SMS test-number sign-in, invalid/expired code, resend and cancel; otherwise inspect the unavailable-provider state.</x:v>
+      </x:c>
+      <x:c r="G156" s="9" t="str">
+        <x:v>Only configured providers work; errors and retry limits are clear and cancellation grants no session. A disabled provider is not falsely reported as tested.</x:v>
+      </x:c>
+      <x:c r="H156" s="9" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
+      <x:c r="I156" s="12" t="str"/>
+      <x:c r="J156" s="12" t="str"/>
+      <x:c r="K156" s="12" t="str"/>
+      <x:c r="L156" s="13"/>
+      <x:c r="M156" s="9" t="str">
+        <x:v>Use Firebase test numbers or an authorized disposable recipient; no real staff SMS.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:M2"/>
@@ -5242,7 +5473,7 @@
     <x:mergeCell ref="K4:M4"/>
     <x:mergeCell ref="A5:M5"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="H9:H149">
+  <x:conditionalFormatting sqref="H9:H156">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <x:formula>"Fail"</x:formula>
     </x:cfRule>
@@ -5257,13 +5488,13 @@
     <x:dataValidation type="list" sqref="H3">
       <x:formula1>"Frontend Demo,Firebase Lab,Isolated backend"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="H9:H149">
+    <x:dataValidation type="list" sqref="H9:H156">
       <x:formula1>"Not run,Pass,Fail,Blocked,N/A"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe571fc527ac415f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86710499bf73415b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>